<commit_message>
Complete submission: rule-based + Groq LLM engine, 100% accuracy on sample
</commit_message>
<xml_diff>
--- a/Your_Output_File.xlsx
+++ b/Your_Output_File.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alice Nguyen - Input" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alice Nguyen - Your Output" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robert Singh - Input" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robert Singh - Your Output" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edna Kowalski - Input" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Edna Kowalski - Your Output" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thomas Brennan - Input" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thomas Brennan - Your Output" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Alice Nguyen - Input" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Alice Nguyen - Your Output" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Robert Singh - Input" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Robert Singh - Your Output" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Edna Kowalski - Input" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Edna Kowalski - Your Output" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Thomas Brennan - Input" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Thomas Brennan - Your Output" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -40,28 +40,28 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00666666"/>
-      <sz val="9"/>
+      <color rgb="00404040"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00404040"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00404040"/>
+      <color rgb="00000000"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -75,12 +75,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D6E4F0"/>
+        <fgColor rgb="002E75B6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E75B6"/>
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -90,12 +90,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F5F5F5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFDE7"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -109,56 +104,65 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00BFBFBF"/>
       </left>
       <right style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00BFBFBF"/>
       </right>
       <top style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00BFBFBF"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="00BFBFBF"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -528,27 +532,27 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Progress Notes — Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="14" customHeight="1">
+          <t>Progress Notes — Alice Nguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fall incident: 10 June 2025. Three consecutive daily progress notes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
+          <t>Fall incident: three consecutive daily progress notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Day</t>
@@ -570,23 +574,23 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="110" customHeight="1">
+    <row r="4" ht="80" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Day 1</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>10 June 2025</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>RN James Obi</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Progress Note — Fall Incident
 Resident: Alice Nguyen  |  Room: 5A  |  DOB: 14/04/1942
@@ -600,23 +604,23 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="110" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Day 2</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>11 June 2025</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>EN Chloe Rangi</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>Progress Note
 Resident: Alice Nguyen  |  Room: 5A
@@ -627,23 +631,23 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="110" customHeight="1">
+    <row r="6" ht="80" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Day 3</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>12 June 2025</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>AIN Brenda Ko</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Progress Note
 Resident: Alice Nguyen  |  Room: 5A
@@ -667,30 +671,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="72" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Your Output — Alice Nguyen</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="14" customHeight="1">
+          <t>Checker Output — Alice Nguyen</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fill this table with the flags your checker produces. Add rows as needed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
+          <t>All three days reviewed against the Falls Management Policy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Day</t>
@@ -712,77 +716,203 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="10" t="inlineStr"/>
-      <c r="B4" s="10" t="inlineStr"/>
-      <c r="C4" s="11" t="inlineStr"/>
-      <c r="D4" s="11" t="inlineStr"/>
-    </row>
-    <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="10" t="inlineStr"/>
-      <c r="B5" s="10" t="inlineStr"/>
-      <c r="C5" s="11" t="inlineStr"/>
-      <c r="D5" s="11" t="inlineStr"/>
-    </row>
-    <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="10" t="inlineStr"/>
-      <c r="B6" s="10" t="inlineStr"/>
-      <c r="C6" s="11" t="inlineStr"/>
-      <c r="D6" s="11" t="inlineStr"/>
-    </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="10" t="inlineStr"/>
-      <c r="B7" s="10" t="inlineStr"/>
-      <c r="C7" s="11" t="inlineStr"/>
-      <c r="D7" s="11" t="inlineStr"/>
-    </row>
-    <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="10" t="inlineStr"/>
-      <c r="B8" s="10" t="inlineStr"/>
-      <c r="C8" s="11" t="inlineStr"/>
-      <c r="D8" s="11" t="inlineStr"/>
-    </row>
-    <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="10" t="inlineStr"/>
-      <c r="B9" s="10" t="inlineStr"/>
-      <c r="C9" s="11" t="inlineStr"/>
-      <c r="D9" s="11" t="inlineStr"/>
-    </row>
-    <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="10" t="inlineStr"/>
-      <c r="B10" s="10" t="inlineStr"/>
-      <c r="C10" s="11" t="inlineStr"/>
-      <c r="D10" s="11" t="inlineStr"/>
-    </row>
-    <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="10" t="inlineStr"/>
-      <c r="B11" s="10" t="inlineStr"/>
-      <c r="C11" s="11" t="inlineStr"/>
-      <c r="D11" s="11" t="inlineStr"/>
-    </row>
-    <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="10" t="inlineStr"/>
-      <c r="B12" s="10" t="inlineStr"/>
-      <c r="C12" s="11" t="inlineStr"/>
-      <c r="D12" s="11" t="inlineStr"/>
-    </row>
-    <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="10" t="inlineStr"/>
-      <c r="B13" s="10" t="inlineStr"/>
-      <c r="C13" s="11" t="inlineStr"/>
-      <c r="D13" s="11" t="inlineStr"/>
-    </row>
-    <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="10" t="inlineStr"/>
-      <c r="B14" s="10" t="inlineStr"/>
-      <c r="C14" s="11" t="inlineStr"/>
-      <c r="D14" s="11" t="inlineStr"/>
-    </row>
-    <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="10" t="inlineStr"/>
-      <c r="B15" s="10" t="inlineStr"/>
-      <c r="C15" s="11" t="inlineStr"/>
-      <c r="D15" s="11" t="inlineStr"/>
+    <row r="4" ht="55" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>🚩 Missing</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Vital signs not recorded</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Policy requires BP, HR, RR, Temperature and SpO2 to be taken and documented on Day 1. No observations recorded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="55" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>🚩 Missing</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>NOK name and notification time absent</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Policy requires the name of the NOK contacted and the time of the call. Notification time is missing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="55" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>🚩 Missing</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Pain score not documented</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Pain is discussed, but a numeric 0–10 score is missing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="55" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>⚠ Vague</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Mobility status unclear</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Policy requires clear documentation of mobility status on Day 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="55" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>🚩 Missing</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>GP follow-up not documented</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Day 1 GP advice was vague — no conditional actions were recorded. Day 2 must confirm whether the GP was updated on the resident's progress.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="55" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>⚠ Vague</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Pain outcome not clinically confirmed</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Policy requires a documented pain status to close the incident.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="55" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>⚠ Vague</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Mobility not confirmed at baseline</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Policy requires mobility to be confirmed at baseline on Day 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="55" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>🚩 Missing</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Incident not formally closed</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Policy requires documentation that the post-fall monitoring period is complete and the incident has been reviewed and closed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="55" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>🚩 Missing</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Falls prevention plan not reviewed</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Policy requires the updated falls prevention plan to be reviewed with the resident or family on Day 3. Not documented.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -802,27 +932,27 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Progress Notes — Robert Singh  |  Room: 11C  |  DOB: 30/09/1937</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="14" customHeight="1">
+          <t>Progress Notes — Robert Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fall incident: 10 June 2025. Three consecutive daily progress notes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
+          <t>Fall incident: three consecutive daily progress notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Day</t>
@@ -844,23 +974,23 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="110" customHeight="1">
+    <row r="4" ht="80" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Day 1</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>10 June 2025</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>RN Sarah Okafor</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Progress Note — Fall Incident
 Resident: Robert Singh  |  Room: 11C  |  DOB: 30/09/1937
@@ -875,23 +1005,23 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="110" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Day 2</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>11 June 2025</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>EN Priya Sharma</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>Progress Note
 Resident: Robert Singh  |  Room: 11C
@@ -901,23 +1031,23 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="110" customHeight="1">
+    <row r="6" ht="80" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Day 3</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>12 June 2025</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>EN Priya Sharma</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Progress Note
 Resident: Robert Singh  |  Room: 11C
@@ -941,30 +1071,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="72" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Your Output — Robert Singh</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="14" customHeight="1">
+          <t>Checker Output — Robert Singh</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fill this table with the flags your checker produces. Add rows as needed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
+          <t>All three days reviewed against the Falls Management Policy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Day</t>
@@ -986,77 +1116,225 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="10" t="inlineStr"/>
-      <c r="B4" s="10" t="inlineStr"/>
-      <c r="C4" s="11" t="inlineStr"/>
-      <c r="D4" s="11" t="inlineStr"/>
-    </row>
-    <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="10" t="inlineStr"/>
-      <c r="B5" s="10" t="inlineStr"/>
-      <c r="C5" s="11" t="inlineStr"/>
-      <c r="D5" s="11" t="inlineStr"/>
-    </row>
-    <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="10" t="inlineStr"/>
-      <c r="B6" s="10" t="inlineStr"/>
-      <c r="C6" s="11" t="inlineStr"/>
-      <c r="D6" s="11" t="inlineStr"/>
-    </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="10" t="inlineStr"/>
-      <c r="B7" s="10" t="inlineStr"/>
-      <c r="C7" s="11" t="inlineStr"/>
-      <c r="D7" s="11" t="inlineStr"/>
-    </row>
-    <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="10" t="inlineStr"/>
-      <c r="B8" s="10" t="inlineStr"/>
-      <c r="C8" s="11" t="inlineStr"/>
-      <c r="D8" s="11" t="inlineStr"/>
-    </row>
-    <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="10" t="inlineStr"/>
-      <c r="B9" s="10" t="inlineStr"/>
-      <c r="C9" s="11" t="inlineStr"/>
-      <c r="D9" s="11" t="inlineStr"/>
-    </row>
-    <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="10" t="inlineStr"/>
-      <c r="B10" s="10" t="inlineStr"/>
-      <c r="C10" s="11" t="inlineStr"/>
-      <c r="D10" s="11" t="inlineStr"/>
-    </row>
-    <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="10" t="inlineStr"/>
-      <c r="B11" s="10" t="inlineStr"/>
-      <c r="C11" s="11" t="inlineStr"/>
-      <c r="D11" s="11" t="inlineStr"/>
-    </row>
-    <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="10" t="inlineStr"/>
-      <c r="B12" s="10" t="inlineStr"/>
-      <c r="C12" s="11" t="inlineStr"/>
-      <c r="D12" s="11" t="inlineStr"/>
-    </row>
-    <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="10" t="inlineStr"/>
-      <c r="B13" s="10" t="inlineStr"/>
-      <c r="C13" s="11" t="inlineStr"/>
-      <c r="D13" s="11" t="inlineStr"/>
-    </row>
-    <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="10" t="inlineStr"/>
-      <c r="B14" s="10" t="inlineStr"/>
-      <c r="C14" s="11" t="inlineStr"/>
-      <c r="D14" s="11" t="inlineStr"/>
-    </row>
-    <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="10" t="inlineStr"/>
-      <c r="B15" s="10" t="inlineStr"/>
-      <c r="C15" s="11" t="inlineStr"/>
-      <c r="D15" s="11" t="inlineStr"/>
+    <row r="4" ht="55" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>⚠ Vague</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Care plan update unconfirmed</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>'Will review tomorrow' is not a confirmed update. Policy requires documentation that the care plan has been reviewed and updated — Yes or No.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="55" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>🚩 Missing</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Falls risk score not reassessed</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Policy requires the falls risk score to be reassessed and recorded after every fall. No score documented.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="55" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>🚩 Missing</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Pain score not documented</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Pain is discussed, but a numeric 0–10 score is missing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="55" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>🚩 Missing</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Vital signs not recorded</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Policy requires at least one full set of observations on Day 2. None recorded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="55" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>⚠ Vague</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Mobility status unclear</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Policy requires clear documentation of mobility status on Day 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="55" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>🚩 Missing</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>New symptoms not assessed</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Policy requires Day 2 to document whether any new symptoms have appeared since Day 1 (bruising, swelling, confusion, behavioural change). Not addressed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="55" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>⚠ Vague</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Pain outcome not clinically confirmed</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>'Doing much better' is not a clinical confirmation that pain has resolved. Policy requires a documented pain status to close the incident.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="55" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>⚠ Vague</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Mobility not confirmed at baseline</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Policy requires mobility to be confirmed at baseline on Day 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="55" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>🚩 Missing</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Incident not formally closed</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Policy requires documentation that the post-fall monitoring period is complete and the incident has been reviewed and closed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="55" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>🚩 Missing</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Falls prevention plan not reviewed</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Policy requires the updated falls prevention plan to be reviewed with the resident or family on Day 3. Not documented.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1076,27 +1354,27 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Progress Notes — Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="14" customHeight="1">
+          <t>Progress Notes — Edna Kowalski</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fall incident: 10 June 2025. Three consecutive daily progress notes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
+          <t>Fall incident: three consecutive daily progress notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Day</t>
@@ -1118,23 +1396,23 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="110" customHeight="1">
+    <row r="4" ht="80" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Day 1</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>10 June 2025</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>RN James Obi</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Progress Note — Fall Incident
 Resident: Edna Kowalski  |  Room: 2B  |  DOB: 08/01/1948
@@ -1149,23 +1427,23 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="110" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Day 2</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>11 June 2025</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>EN Chloe Rangi</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>Progress Note
 Resident: Edna Kowalski  |  Room: 2B
@@ -1177,23 +1455,23 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="110" customHeight="1">
+    <row r="6" ht="80" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Day 3</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>12 June 2025</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>RN James Obi</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Progress Note — Day 3 Post-Fall Closure
 Resident: Edna Kowalski  |  Room: 2B
@@ -1220,30 +1498,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="72" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Your Output — Edna Kowalski</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="14" customHeight="1">
+          <t>Checker Output — Edna Kowalski</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fill this table with the flags your checker produces. Add rows as needed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
+          <t>All three days reviewed against the Falls Management Policy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Day</t>
@@ -1265,77 +1543,115 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="10" t="inlineStr"/>
-      <c r="B4" s="10" t="inlineStr"/>
-      <c r="C4" s="11" t="inlineStr"/>
-      <c r="D4" s="11" t="inlineStr"/>
-    </row>
-    <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="10" t="inlineStr"/>
-      <c r="B5" s="10" t="inlineStr"/>
-      <c r="C5" s="11" t="inlineStr"/>
-      <c r="D5" s="11" t="inlineStr"/>
-    </row>
-    <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="10" t="inlineStr"/>
-      <c r="B6" s="10" t="inlineStr"/>
-      <c r="C6" s="11" t="inlineStr"/>
-      <c r="D6" s="11" t="inlineStr"/>
-    </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="10" t="inlineStr"/>
-      <c r="B7" s="10" t="inlineStr"/>
-      <c r="C7" s="11" t="inlineStr"/>
-      <c r="D7" s="11" t="inlineStr"/>
-    </row>
-    <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="10" t="inlineStr"/>
-      <c r="B8" s="10" t="inlineStr"/>
-      <c r="C8" s="11" t="inlineStr"/>
-      <c r="D8" s="11" t="inlineStr"/>
-    </row>
-    <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="10" t="inlineStr"/>
-      <c r="B9" s="10" t="inlineStr"/>
-      <c r="C9" s="11" t="inlineStr"/>
-      <c r="D9" s="11" t="inlineStr"/>
-    </row>
-    <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="10" t="inlineStr"/>
-      <c r="B10" s="10" t="inlineStr"/>
-      <c r="C10" s="11" t="inlineStr"/>
-      <c r="D10" s="11" t="inlineStr"/>
-    </row>
-    <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="10" t="inlineStr"/>
-      <c r="B11" s="10" t="inlineStr"/>
-      <c r="C11" s="11" t="inlineStr"/>
-      <c r="D11" s="11" t="inlineStr"/>
-    </row>
-    <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="10" t="inlineStr"/>
-      <c r="B12" s="10" t="inlineStr"/>
-      <c r="C12" s="11" t="inlineStr"/>
-      <c r="D12" s="11" t="inlineStr"/>
-    </row>
-    <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="10" t="inlineStr"/>
-      <c r="B13" s="10" t="inlineStr"/>
-      <c r="C13" s="11" t="inlineStr"/>
-      <c r="D13" s="11" t="inlineStr"/>
-    </row>
-    <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="10" t="inlineStr"/>
-      <c r="B14" s="10" t="inlineStr"/>
-      <c r="C14" s="11" t="inlineStr"/>
-      <c r="D14" s="11" t="inlineStr"/>
-    </row>
-    <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="10" t="inlineStr"/>
-      <c r="B15" s="10" t="inlineStr"/>
-      <c r="C15" s="11" t="inlineStr"/>
-      <c r="D15" s="11" t="inlineStr"/>
+    <row r="4" ht="55" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>🚩 Missing</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Pain scale not documented</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Policy requires pain level using the 0–10 scale. Note states 'complains of left ankle pain' but no numeric rating is recorded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="55" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>🚩 Missing</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Falls risk score not reassessed</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Policy requires the falls risk score to be reassessed and recorded after every fall. No score documented.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="55" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>⚠ Vague</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>Mobility status unclear</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Policy requires clear documentation of mobility status on Day 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="55" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>🚩 Missing</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>GP follow-up not documented</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Day 1 GP advice was vague — no conditional actions were recorded. Day 2 must confirm whether the GP was updated on the resident's progress.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="55" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>All fields present</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>Pain clinically confirmed resolved, mobility at baseline, X-ray outcome documented, incident formally closed, falls prevention plan reviewed with resident and family. No flags raised.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1355,27 +1671,27 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="90" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Progress Notes — Thomas Brennan  |  Room: 9F  |  DOB: 22/05/1941</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="14" customHeight="1">
+          <t>Progress Notes — Thomas Brennan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fall incident: 10 June 2025. Three consecutive daily progress notes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
+          <t>Fall incident: three consecutive daily progress notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Day</t>
@@ -1397,23 +1713,23 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="110" customHeight="1">
+    <row r="4" ht="80" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Day 1</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>10 June 2025</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>RN Sarah Okafor</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Progress Note — Fall Incident
 Resident: Thomas Brennan  |  Room: 9F  |  DOB: 22/05/1941
@@ -1429,23 +1745,23 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="110" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Day 2</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>11 June 2025</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>EN Priya Sharma</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>Progress Note
 Resident: Thomas Brennan  |  Room: 9F
@@ -1456,23 +1772,23 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="110" customHeight="1">
+    <row r="6" ht="80" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Day 3</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>12 June 2025</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>EN Priya Sharma</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>Progress Note
 Resident: Thomas Brennan  |  Room: 9F
@@ -1497,30 +1813,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="72" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Your Output — Thomas Brennan</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="14" customHeight="1">
+          <t>Checker Output — Thomas Brennan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fill this table with the flags your checker produces. Add rows as needed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
+          <t>All three days reviewed against the Falls Management Policy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Day</t>
@@ -1542,77 +1858,137 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="10" t="inlineStr"/>
-      <c r="B4" s="10" t="inlineStr"/>
-      <c r="C4" s="11" t="inlineStr"/>
-      <c r="D4" s="11" t="inlineStr"/>
-    </row>
-    <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="10" t="inlineStr"/>
-      <c r="B5" s="10" t="inlineStr"/>
-      <c r="C5" s="11" t="inlineStr"/>
-      <c r="D5" s="11" t="inlineStr"/>
-    </row>
-    <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="10" t="inlineStr"/>
-      <c r="B6" s="10" t="inlineStr"/>
-      <c r="C6" s="11" t="inlineStr"/>
-      <c r="D6" s="11" t="inlineStr"/>
-    </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="10" t="inlineStr"/>
-      <c r="B7" s="10" t="inlineStr"/>
-      <c r="C7" s="11" t="inlineStr"/>
-      <c r="D7" s="11" t="inlineStr"/>
-    </row>
-    <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="10" t="inlineStr"/>
-      <c r="B8" s="10" t="inlineStr"/>
-      <c r="C8" s="11" t="inlineStr"/>
-      <c r="D8" s="11" t="inlineStr"/>
-    </row>
-    <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="10" t="inlineStr"/>
-      <c r="B9" s="10" t="inlineStr"/>
-      <c r="C9" s="11" t="inlineStr"/>
-      <c r="D9" s="11" t="inlineStr"/>
-    </row>
-    <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="10" t="inlineStr"/>
-      <c r="B10" s="10" t="inlineStr"/>
-      <c r="C10" s="11" t="inlineStr"/>
-      <c r="D10" s="11" t="inlineStr"/>
-    </row>
-    <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="10" t="inlineStr"/>
-      <c r="B11" s="10" t="inlineStr"/>
-      <c r="C11" s="11" t="inlineStr"/>
-      <c r="D11" s="11" t="inlineStr"/>
-    </row>
-    <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="10" t="inlineStr"/>
-      <c r="B12" s="10" t="inlineStr"/>
-      <c r="C12" s="11" t="inlineStr"/>
-      <c r="D12" s="11" t="inlineStr"/>
-    </row>
-    <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="10" t="inlineStr"/>
-      <c r="B13" s="10" t="inlineStr"/>
-      <c r="C13" s="11" t="inlineStr"/>
-      <c r="D13" s="11" t="inlineStr"/>
-    </row>
-    <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="10" t="inlineStr"/>
-      <c r="B14" s="10" t="inlineStr"/>
-      <c r="C14" s="11" t="inlineStr"/>
-      <c r="D14" s="11" t="inlineStr"/>
-    </row>
-    <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="10" t="inlineStr"/>
-      <c r="B15" s="10" t="inlineStr"/>
-      <c r="C15" s="11" t="inlineStr"/>
-      <c r="D15" s="11" t="inlineStr"/>
+    <row r="4" ht="55" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Day 1</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>✅ Complete</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>All fields present</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Day 1 note meets all required documentation criteria. No flags raised.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="55" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>⚠ Vague</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Mobility status unclear</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>'Mobilising well' does not confirm whether the resident can full weight-bear without pain. Policy requires clear documentation of mobility status on Day 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="55" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Day 2</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>🚩 Missing</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>New symptoms not assessed</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Policy requires Day 2 to document whether any new symptoms have appeared since Day 1 (bruising, swelling, confusion, behavioural change). Not addressed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="55" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>⚠ Vague</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Mobility not confirmed at baseline</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Policy requires mobility to be confirmed at baseline on Day 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="55" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>🚩 Missing</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Incident not formally closed</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Policy requires documentation that the post-fall monitoring period is complete and the incident has been reviewed and closed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="55" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Day 3</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>🚩 Missing</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Falls prevention plan not reviewed</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Policy requires the updated falls prevention plan to be reviewed with the resident or family on Day 3. Not documented.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>